<commit_message>
Updated project Excel sheets (Sprint Backlog, Unit Tests, Defect Tracker, Retrospective)
</commit_message>
<xml_diff>
--- a/Defect_Tracker_IRCTC_IVR.xlsx
+++ b/Defect_Tracker_IRCTC_IVR.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/ad8e6a89a6abcdc6/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/ad8e6a89a6abcdc6/Desktop/Infosys/IRCTC-Conversational-IVR-Modernization-Framework/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10" documentId="8_{F1E83827-CB56-4580-B50A-6F08BDBD4987}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{59EF1569-4FFB-4CE7-8396-B166BFBD4585}"/>
+  <xr:revisionPtr revIDLastSave="62" documentId="8_{F1E83827-CB56-4580-B50A-6F08BDBD4987}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FA97D574-B12C-4010-8DD4-996083167A14}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="66">
   <si>
     <t>Sl No</t>
   </si>
@@ -76,60 +76,24 @@
     <t>Backend Team</t>
   </si>
   <si>
-    <t>VXML parser returning incorrect next state 'agent' when user selects option 5; middleware not handling agent state</t>
-  </si>
-  <si>
-    <t>Added explicit agent-state handler in middleware; resets to menu after response</t>
-  </si>
-  <si>
-    <t>State machine diagram updated in docs</t>
-  </si>
-  <si>
     <t>Sprint 2</t>
   </si>
   <si>
     <t>Performance</t>
   </si>
   <si>
-    <t>Keyword mapper routing 'train availability' query to ticket booking flow instead of availability flow</t>
-  </si>
-  <si>
-    <t>Reordered conditional checks in detect_voice_option(); availability checked before booking</t>
-  </si>
-  <si>
-    <t>All keyword routing unit tests now passing</t>
-  </si>
-  <si>
     <t>Sprint 3</t>
   </si>
   <si>
     <t>Compatibility</t>
   </si>
   <si>
-    <t>Bot hearing its own TTS voice output and sending it back as user input causing infinite response loop</t>
-  </si>
-  <si>
     <t>Logic / UX</t>
   </si>
   <si>
-    <t>Added isSpeaking flag; stopVoice() called before TTS; mic restarts only in speak() onend callback</t>
-  </si>
-  <si>
-    <t>Voice loop fully resolved; tested over 20 cycles</t>
-  </si>
-  <si>
-    <t>Booking flow state machine resetting to menu after first input (source station) instead of advancing to destination</t>
-  </si>
-  <si>
     <t>Sprint 4</t>
   </si>
   <si>
-    <t>Fixed state transition in middleware; 'source' state now correctly updates to 'destination'</t>
-  </si>
-  <si>
-    <t>All booking flow steps verified end-to-end</t>
-  </si>
-  <si>
     <t>Configuration</t>
   </si>
   <si>
@@ -143,6 +107,123 @@
   </si>
   <si>
     <t>Others</t>
+  </si>
+  <si>
+    <t>VXML parser returning incorrect next state when selecting option 5 (agent flow issue)</t>
+  </si>
+  <si>
+    <t>Added explicit agent → menu reset logic in middleware</t>
+  </si>
+  <si>
+    <t>State transition corrected and verified</t>
+  </si>
+  <si>
+    <t>Keyword mapping routing 'train availability' to booking flow</t>
+  </si>
+  <si>
+    <t>Reordered condition checks to prioritize availability</t>
+  </si>
+  <si>
+    <t>13/02/2026</t>
+  </si>
+  <si>
+    <t>All routing tests passed</t>
+  </si>
+  <si>
+    <t>18/02/2026</t>
+  </si>
+  <si>
+    <t>Bot capturing its own TTS voice causing infinite loop</t>
+  </si>
+  <si>
+    <t>Added isSpeaking flag and muted mic during speech</t>
+  </si>
+  <si>
+    <t>19/02/2026</t>
+  </si>
+  <si>
+    <t>Voice loop resolved successfully</t>
+  </si>
+  <si>
+    <t>24/02/2026</t>
+  </si>
+  <si>
+    <t>Booking flow resetting to menu after source station input</t>
+  </si>
+  <si>
+    <t>Fixed middleware state transition (source → destination)</t>
+  </si>
+  <si>
+    <t>25/02/2026</t>
+  </si>
+  <si>
+    <t>Booking flow working correctly</t>
+  </si>
+  <si>
+    <t>29/03/2026</t>
+  </si>
+  <si>
+    <t>Start button not triggering IVR interface</t>
+  </si>
+  <si>
+    <t>UI / Logic</t>
+  </si>
+  <si>
+    <t>Fixed DOM loading and event binding issue</t>
+  </si>
+  <si>
+    <t>Start button working properly</t>
+  </si>
+  <si>
+    <t>30/03/2026</t>
+  </si>
+  <si>
+    <t>Welcome message not speaking automatically</t>
+  </si>
+  <si>
+    <t>Voice / UX</t>
+  </si>
+  <si>
+    <t>Handled browser autoplay restriction using user interaction</t>
+  </si>
+  <si>
+    <t>Voice output working after interaction</t>
+  </si>
+  <si>
+    <t>Cancel ticket voice command mapped incorrectly to booking</t>
+  </si>
+  <si>
+    <t>Reordered intent detection conditions</t>
+  </si>
+  <si>
+    <t>Cancel ticket detection fixed</t>
+  </si>
+  <si>
+    <t>Voice recognition stopping after one response</t>
+  </si>
+  <si>
+    <t>Voice / Logic</t>
+  </si>
+  <si>
+    <t>Added auto restart of speech recognition</t>
+  </si>
+  <si>
+    <t>Continuous voice interaction working</t>
+  </si>
+  <si>
+    <t>IVR not starting automatically after UI load</t>
+  </si>
+  <si>
+    <t>Integration</t>
+  </si>
+  <si>
+    <t>Added API call on IVR start</t>
+  </si>
+  <si>
+    <t>IVR auto start working</t>
+  </si>
+  <si>
+    <t>Voice / Speech</t>
   </si>
 </sst>
 </file>
@@ -152,7 +233,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -170,6 +251,12 @@
     <font>
       <sz val="10"/>
       <name val="Arial"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <charset val="1"/>
     </font>
   </fonts>
@@ -234,7 +321,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -503,21 +590,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K5"/>
+  <dimension ref="A1:K10"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="7" customWidth="1"/>
-    <col min="2" max="3" width="14" customWidth="1"/>
-    <col min="4" max="4" width="52" customWidth="1"/>
+    <col min="2" max="2" width="15.77734375" customWidth="1"/>
+    <col min="3" max="3" width="15.44140625" customWidth="1"/>
+    <col min="4" max="4" width="91.21875" customWidth="1"/>
     <col min="5" max="5" width="14" customWidth="1"/>
     <col min="6" max="7" width="16" customWidth="1"/>
-    <col min="8" max="8" width="52" customWidth="1"/>
-    <col min="9" max="9" width="16" customWidth="1"/>
+    <col min="8" max="8" width="70.5546875" customWidth="1"/>
+    <col min="9" max="9" width="63" customWidth="1"/>
     <col min="10" max="10" width="18" customWidth="1"/>
-    <col min="11" max="11" width="30" customWidth="1"/>
+    <col min="11" max="11" width="45" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -552,7 +640,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="36" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:11" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -560,10 +648,10 @@
         <v>15</v>
       </c>
       <c r="C2" s="3">
-        <v>46060</v>
+        <v>46205</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>16</v>
+        <v>27</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>12</v>
@@ -575,19 +663,19 @@
         <v>13</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>17</v>
+        <v>28</v>
       </c>
       <c r="I2" s="3">
-        <v>46061</v>
+        <v>46236</v>
       </c>
       <c r="J2" s="2" t="s">
         <v>14</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" ht="36" customHeight="1" x14ac:dyDescent="0.3">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="2">
         <v>2</v>
       </c>
@@ -595,13 +683,13 @@
         <v>15</v>
       </c>
       <c r="C3" s="3">
-        <v>46065</v>
+        <v>46358</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="F3" s="2" t="s">
         <v>15</v>
@@ -610,68 +698,68 @@
         <v>13</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="I3" s="3">
-        <v>46066</v>
+        <v>31</v>
+      </c>
+      <c r="I3" s="3" t="s">
+        <v>32</v>
       </c>
       <c r="J3" s="2" t="s">
         <v>14</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" ht="36" customHeight="1" x14ac:dyDescent="0.3">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="2">
         <v>3</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C4" s="3">
-        <v>46071</v>
+      <c r="C4" s="3" t="s">
+        <v>34</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="F4" s="2" t="s">
         <v>11</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="I4" s="3">
-        <v>46072</v>
+        <v>36</v>
+      </c>
+      <c r="I4" s="3" t="s">
+        <v>37</v>
       </c>
       <c r="J4" s="2" t="s">
         <v>14</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" ht="36" customHeight="1" x14ac:dyDescent="0.3">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2">
         <v>4</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C5" s="3">
-        <v>46077</v>
+      <c r="C5" s="3" t="s">
+        <v>39</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="F5" s="2" t="s">
         <v>15</v>
@@ -680,19 +768,195 @@
         <v>13</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="I5" s="3">
-        <v>46078</v>
+        <v>41</v>
+      </c>
+      <c r="I5" s="3" t="s">
+        <v>42</v>
       </c>
       <c r="J5" s="2" t="s">
         <v>14</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>33</v>
+        <v>43</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="2">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="I6" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="J6" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="K6" s="2" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="2">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="I7" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="J7" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="K7" s="2" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="2">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="I8" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="J8" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="K8" s="2" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="2">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="I9" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="J9" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="K9" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="2">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="I10" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="J10" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="K10" s="2" t="s">
+        <v>64</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
@@ -700,8 +964,11 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:A11"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="17.6640625" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:1" ht="23.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
@@ -713,39 +980,49 @@
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A4" s="5" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A5" s="5" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A6" s="5" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A7" s="5" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A8" s="5" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A9" s="5" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="6" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="5" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="5" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="8" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="5" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="9" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="5" t="s">
-        <v>38</v>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A10" s="5" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A11" s="5" t="s">
+        <v>26</v>
       </c>
     </row>
   </sheetData>

</xml_diff>